<commit_message>
add: tambah jenis soal benar salah menggantikan soal uraian singkat
</commit_message>
<xml_diff>
--- a/public/Template_Soal.xlsx
+++ b/public/Template_Soal.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="PG" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="PG Kompleks" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Menjodohkan" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Esai" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Benar Salah" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Teks_Soal</t>
   </si>
@@ -112,16 +113,27 @@
   </si>
   <si>
     <t xml:space="preserve">Visi: Maju bersama... Misi: 1. ... 2. ...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Javascript adalah bahasa pemrograman</t>
+  </si>
+  <si>
+    <t>BENAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ibukota negara Indonesia saat ini adalah Bandung</t>
+  </si>
+  <si>
+    <t>SALAH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.000000"/>
-      <color indexed="64"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -132,13 +144,16 @@
     <font>
       <b/>
       <sz val="12.000000"/>
-      <color indexed="64"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12.000000"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="12.000000"/>
       <color indexed="64"/>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
     </font>
   </fonts>
   <fills count="2">
@@ -159,16 +174,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
@@ -176,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -193,6 +208,9 @@
       <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -972,4 +990,73 @@
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="45.57421875"/>
+    <col bestFit="1" min="7" max="7" width="13.8515625"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="12.75">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" ht="12.75">
+      <c r="A2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" ht="15">
+      <c r="A3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>